<commit_message>
picking_items line ids + sync_events table-change feed
- picking_items: add line_id / line_number / shipment_number (required on
  ingest, reconciled by part_no) and backend-maintained line status
  (pending/picked); surfaced on PDA picking detail + scan pages and the
  admin order detail; seed workbook + generator updated
- sync_events: trigger-written table-change feed for the external sync
  service — sync_events_notify() on every business table, only commits by
  the warehouse role recorded (warehouse_sync skipped, breaking the
  circular-event loop), seed/reset suppressed via app.sync_events_off
- GET /sync-events?since= poll endpoint; warehouse_sync role created in
  the migration + prod compose init script (SYNC_DB_PASSWORD)
- docs: sync event catalog, schema tables, ingest payload notes
</commit_message>
<xml_diff>
--- a/new_seed/demo-scenario.xlsx
+++ b/new_seed/demo-scenario.xlsx
@@ -1145,7 +1145,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1157,6 +1157,15 @@
       <c r="C1" t="str">
         <v>qty</v>
       </c>
+      <c r="D1" t="str">
+        <v>lineId</v>
+      </c>
+      <c r="E1" t="str">
+        <v>lineNumber</v>
+      </c>
+      <c r="F1" t="str">
+        <v>shipmentNumber</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1168,6 +1177,15 @@
       <c r="C2">
         <v>1000</v>
       </c>
+      <c r="D2">
+        <v>1001</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1179,6 +1197,15 @@
       <c r="C3">
         <v>500</v>
       </c>
+      <c r="D3">
+        <v>1002</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1190,6 +1217,15 @@
       <c r="C4">
         <v>1000</v>
       </c>
+      <c r="D4">
+        <v>2001</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1201,6 +1237,15 @@
       <c r="C5">
         <v>600</v>
       </c>
+      <c r="D5">
+        <v>2002</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1212,10 +1257,39 @@
       <c r="C6">
         <v>700</v>
       </c>
+      <c r="D6">
+        <v>2003</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>SO-DEMO-0001</v>
+      </c>
+      <c r="B7" t="str">
+        <v>RK73B1JTTD181G</v>
+      </c>
+      <c r="C7">
+        <v>300</v>
+      </c>
+      <c r="D7">
+        <v>1003</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1375,7 +1449,7 @@
         <v>RK73B1JTTD181G</v>
       </c>
       <c r="D4">
-        <v>400</v>
+        <v>700</v>
       </c>
       <c r="E4" t="str">
         <v>2604</v>

</xml_diff>

<commit_message>
seed: three allocation demo cases on receiving 100003 (exact carton / under-supplied / split)
</commit_message>
<xml_diff>
--- a/new_seed/demo-scenario.xlsx
+++ b/new_seed/demo-scenario.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -466,16 +466,36 @@
         <v>pending</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>100003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>KOA</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-08-03</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="str">
+        <v>STORE1</v>
+      </c>
+      <c r="F4" t="str">
+        <v>pending</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -528,16 +548,33 @@
         <v>2026-07-26</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>100003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>INV-100003-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>KOA</v>
+      </c>
+      <c r="D4" t="str">
+        <v>WCL Components Ltd</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-08-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1056,16 +1093,251 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>INV-100003-01</v>
+      </c>
+      <c r="B12" t="str">
+        <v>C3001</v>
+      </c>
+      <c r="C12" t="str">
+        <v>RK73H1JTTD3302F</v>
+      </c>
+      <c r="D12" t="str">
+        <v>RK73H1JTTD3302F</v>
+      </c>
+      <c r="E12" t="str">
+        <v>PO-KOA-301</v>
+      </c>
+      <c r="F12" t="str">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>500</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2609</v>
+      </c>
+      <c r="I12" t="str">
+        <v>L2609C</v>
+      </c>
+      <c r="J12" t="str">
+        <v>JP</v>
+      </c>
+      <c r="K12" t="str">
+        <v>JP</v>
+      </c>
+      <c r="L12" t="str">
+        <v>30 X 24 X 20</v>
+      </c>
+      <c r="M12">
+        <v>1100</v>
+      </c>
+      <c r="N12">
+        <v>1250</v>
+      </c>
+      <c r="O12" t="str">
+        <v>g</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>INV-100003-01</v>
+      </c>
+      <c r="B13" t="str">
+        <v>C3001</v>
+      </c>
+      <c r="C13" t="str">
+        <v>RK73H1JTTD6802F</v>
+      </c>
+      <c r="D13" t="str">
+        <v>RK73H1JTTD6802F</v>
+      </c>
+      <c r="E13" t="str">
+        <v>PO-KOA-301</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>800</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2609</v>
+      </c>
+      <c r="I13" t="str">
+        <v>L2609D</v>
+      </c>
+      <c r="J13" t="str">
+        <v>JP</v>
+      </c>
+      <c r="K13" t="str">
+        <v>JP</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>INV-100003-01</v>
+      </c>
+      <c r="B14" t="str">
+        <v>C3002</v>
+      </c>
+      <c r="C14" t="str">
+        <v>RK73B1JTTD102G</v>
+      </c>
+      <c r="D14" t="str">
+        <v>RK73B1JTTD102G</v>
+      </c>
+      <c r="E14" t="str">
+        <v>PO-KOA-301</v>
+      </c>
+      <c r="F14" t="str">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>1200</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2610</v>
+      </c>
+      <c r="I14" t="str">
+        <v>L2610A</v>
+      </c>
+      <c r="J14" t="str">
+        <v>JP</v>
+      </c>
+      <c r="K14" t="str">
+        <v>JP</v>
+      </c>
+      <c r="L14" t="str">
+        <v>28 X 20 X 18</v>
+      </c>
+      <c r="M14">
+        <v>800</v>
+      </c>
+      <c r="N14">
+        <v>950</v>
+      </c>
+      <c r="O14" t="str">
+        <v>g</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>INV-100003-01</v>
+      </c>
+      <c r="B15" t="str">
+        <v>C3003</v>
+      </c>
+      <c r="C15" t="str">
+        <v>RK73H1JTTD5602F</v>
+      </c>
+      <c r="D15" t="str">
+        <v>RK73H1JTTD5602F</v>
+      </c>
+      <c r="E15" t="str">
+        <v>PO-KOA-301</v>
+      </c>
+      <c r="F15" t="str">
+        <v>4</v>
+      </c>
+      <c r="G15">
+        <v>1500</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2611</v>
+      </c>
+      <c r="I15" t="str">
+        <v>L2611A</v>
+      </c>
+      <c r="J15" t="str">
+        <v>JP</v>
+      </c>
+      <c r="K15" t="str">
+        <v>JP</v>
+      </c>
+      <c r="L15" t="str">
+        <v>36 X 26 X 24</v>
+      </c>
+      <c r="M15">
+        <v>1900</v>
+      </c>
+      <c r="N15">
+        <v>2100</v>
+      </c>
+      <c r="O15" t="str">
+        <v>g</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>INV-100003-01</v>
+      </c>
+      <c r="B16" t="str">
+        <v>C3003</v>
+      </c>
+      <c r="C16" t="str">
+        <v>RK73H2ATTD2212F</v>
+      </c>
+      <c r="D16" t="str">
+        <v>RK73H2ATTD2212F</v>
+      </c>
+      <c r="E16" t="str">
+        <v>PO-KOA-301</v>
+      </c>
+      <c r="F16" t="str">
+        <v>5</v>
+      </c>
+      <c r="G16">
+        <v>500</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2611</v>
+      </c>
+      <c r="I16" t="str">
+        <v>L2611B</v>
+      </c>
+      <c r="J16" t="str">
+        <v>JP</v>
+      </c>
+      <c r="K16" t="str">
+        <v>JP</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1136,16 +1408,85 @@
         <v>STORE1</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SO-DEMO-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>CUST-PO-9003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-08-04</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ACME Electronics (HK)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>ACME</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" t="str">
+        <v>STORE1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>SO-DEMO-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CUST-PO-9004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-08-05</v>
+      </c>
+      <c r="D5" t="str">
+        <v>ACME Electronics (HK)</v>
+      </c>
+      <c r="E5" t="str">
+        <v>ACME</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" t="str">
+        <v>STORE1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>SO-DEMO-0005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>CUST-PO-9005</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-08-06</v>
+      </c>
+      <c r="D6" t="str">
+        <v>ACME Electronics (HK)</v>
+      </c>
+      <c r="E6" t="str">
+        <v>ACME</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" t="str">
+        <v>STORE1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1209,19 +1550,19 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SO-DEMO-0002</v>
+        <v>SO-DEMO-0001</v>
       </c>
       <c r="B4" t="str">
         <v>RK73B1JTTD181G</v>
       </c>
       <c r="C4">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="D4">
-        <v>2001</v>
+        <v>1003</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1232,16 +1573,16 @@
         <v>SO-DEMO-0002</v>
       </c>
       <c r="B5" t="str">
-        <v>RK73H1JTTD4702F</v>
+        <v>RK73B1JTTD181G</v>
       </c>
       <c r="C5">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="D5">
-        <v>2002</v>
+        <v>2001</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1252,16 +1593,16 @@
         <v>SO-DEMO-0002</v>
       </c>
       <c r="B6" t="str">
-        <v>RK73H2ATTD1372F</v>
+        <v>RK73H1JTTD4702F</v>
       </c>
       <c r="C6">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="D6">
-        <v>2003</v>
+        <v>2002</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -1269,16 +1610,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SO-DEMO-0001</v>
+        <v>SO-DEMO-0002</v>
       </c>
       <c r="B7" t="str">
-        <v>RK73B1JTTD181G</v>
+        <v>RK73H2ATTD1372F</v>
       </c>
       <c r="C7">
-        <v>300</v>
+        <v>700</v>
       </c>
       <c r="D7">
-        <v>1003</v>
+        <v>2003</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -1287,16 +1628,116 @@
         <v>1</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SO-DEMO-0003</v>
+      </c>
+      <c r="B8" t="str">
+        <v>RK73H1JTTD3302F</v>
+      </c>
+      <c r="C8">
+        <v>500</v>
+      </c>
+      <c r="D8">
+        <v>3001</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>SO-DEMO-0003</v>
+      </c>
+      <c r="B9" t="str">
+        <v>RK73H1JTTD6802F</v>
+      </c>
+      <c r="C9">
+        <v>800</v>
+      </c>
+      <c r="D9">
+        <v>3002</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>SO-DEMO-0004</v>
+      </c>
+      <c r="B10" t="str">
+        <v>RK73B1JTTD102G</v>
+      </c>
+      <c r="C10">
+        <v>3000</v>
+      </c>
+      <c r="D10">
+        <v>4001</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>SO-DEMO-0005</v>
+      </c>
+      <c r="B11" t="str">
+        <v>RK73H1JTTD5602F</v>
+      </c>
+      <c r="C11">
+        <v>2500</v>
+      </c>
+      <c r="D11">
+        <v>5001</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>SO-DEMO-0005</v>
+      </c>
+      <c r="B12" t="str">
+        <v>RK73H2ATTD2212F</v>
+      </c>
+      <c r="C12">
+        <v>900</v>
+      </c>
+      <c r="D12">
+        <v>5002</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1349,16 +1790,50 @@
         <v>closed</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>BOX-H-20260701-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>A-02-01</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="str">
+        <v>STORE1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>closed</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>BOX-H-20260701-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>A-02-02</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="str">
+        <v>STORE1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>open</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1490,16 +1965,68 @@
         <v>JP</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>BOX-H-20260701-0003</v>
+      </c>
+      <c r="B6" t="str">
+        <v>A-02-01</v>
+      </c>
+      <c r="C6" t="str">
+        <v>RK73H1JTTD5602F</v>
+      </c>
+      <c r="D6">
+        <v>1000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2609</v>
+      </c>
+      <c r="F6" t="str">
+        <v>L2609A</v>
+      </c>
+      <c r="G6" t="str">
+        <v>JP</v>
+      </c>
+      <c r="H6" t="str">
+        <v>JP</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>BOX-H-20260701-0003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>A-02-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>RK73H2ATTD2212F</v>
+      </c>
+      <c r="D7">
+        <v>400</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2609</v>
+      </c>
+      <c r="F7" t="str">
+        <v>L2609B</v>
+      </c>
+      <c r="G7" t="str">
+        <v>JP</v>
+      </c>
+      <c r="H7" t="str">
+        <v>JP</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1533,47 +2060,117 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Story: 2 pending receiving orders (2 cartons each, 2-3 items per carton),</v>
+        <v>Story: 3 pending receiving orders. 100001/100002 are the original pair:</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PO SO-DEMO-0001 exactly matches shelf box BOX-H-20260701-0001 (whole-box claim),</v>
+        <v>PO SO-DEMO-0001: scan the 181G×300 line item-by-item first — then the</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PO SO-DEMO-0002 is only partially covered by shelf stock — the rest arrives</v>
+        <v>remaining demand exactly matches shelf box BOX-H-20260701-0001 (whole-box claim),</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>on the two receiving orders (process them, then re-allocate).</v>
+        <v>PO SO-DEMO-0002 is only partially covered by shelf stock — the rest arrives</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>on receiving orders 100001/100002 (process them, then re-allocate).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>receiving_items metadata columns boxSize/netWeight/grossWeight/weightUnit</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>are packed into the item's additional_data (weightUnit: g | kg, default kg).</v>
+        <v>100003 feeds the three allocation demo cases:</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>case 1 (SO-DEMO-0003): demand == carton C3001 exactly — receive 100003,</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>then on the picking page scan the C3001 carton label and its two part</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>labels; pack the packages into a new shipping box — its box size/weights</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>prefill from the carton's additional_data and flow to measuring.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>case 2 (SO-DEMO-0004): needs 102G×3000, only 1200 exists (C3002) — the order</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>stays partially allocated on the picking list.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>case 3 (SO-DEMO-0005): both lines split across shelf box BOX-H-20260701-0003</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>and receiving carton C3003.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Print scannable labels (parts, cartons, boxes, shelves) from the web app's</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>/print-labels page (live data from GET /labels-data).</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>receiving_items metadata columns boxSize/netWeight/grossWeight/weightUnit</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>are packed into the item's additional_data (weightUnit: g | kg, default kg).</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>shelf_stock with a blank boxId becomes a loose (unboxed) shelf lot.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>